<commit_message>
Add HLFB muting during tool engagements.
</commit_message>
<xml_diff>
--- a/TCVars_DX200MH180.xlsx
+++ b/TCVars_DX200MH180.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Motoman_EnIP_ToolChanger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013D3007-3427-441C-846A-E9FFDC426908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BED0D09-8C07-4011-ADBF-376F4D27444C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2925" yWindow="1275" windowWidth="24315" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IO Mapping" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="187">
   <si>
     <t>DX200 MH180 - EtherNet/IP Tool Changer I/O Mapping</t>
   </si>
@@ -601,6 +601,18 @@
       </rPr>
       <t>State Machine Bits:  (0=DISABLED, 1=HOMING, 2=IDLE, 3=MOVING, 4=AT_TOOL, 5=FAULTED)</t>
     </r>
+  </si>
+  <si>
+    <t>HLFB Mute Echo</t>
+  </si>
+  <si>
+    <t>True When Output Byte 1, Bit 4 is true.</t>
+  </si>
+  <si>
+    <t>Suppress HLFB out of position faults during pick/put away.</t>
+  </si>
+  <si>
+    <t>Mute HLFB (Tool Engage)</t>
   </si>
 </sst>
 </file>
@@ -739,7 +751,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -769,24 +781,30 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1082,24 +1100,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -1348,22 +1366,24 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="19">
         <v>1</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="19">
         <v>4</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F17" s="5"/>
+      <c r="E17" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
@@ -1584,22 +1604,22 @@
       <c r="F29" s="6"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
     </row>
     <row r="31" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="14" t="s">
+      <c r="A31" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
@@ -1793,7 +1813,7 @@
       <c r="E41" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="F41" s="15" t="s">
+      <c r="F41" s="11" t="s">
         <v>181</v>
       </c>
     </row>
@@ -1927,9 +1947,11 @@
         <v>7</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F48" s="10"/>
+        <v>183</v>
+      </c>
+      <c r="F48" s="10" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
@@ -2566,10 +2588,10 @@
       <c r="F80" s="10"/>
     </row>
     <row r="82" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E82" s="16" t="s">
+      <c r="E82" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="F82" s="16"/>
+      <c r="F82" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>